<commit_message>
Updated rule, test data, results
</commit_message>
<xml_diff>
--- a/rules/CORE-000094/negative/01/data/unit-test-coreid-CG0112-negative.xlsx
+++ b/rules/CORE-000094/negative/01/data/unit-test-coreid-CG0112-negative.xlsx
@@ -1,58 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Library" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
-  </numFmts>
-  <fonts count="4">
+  <numFmts count="0"/>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -62,13 +69,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -76,8 +86,14 @@
         <fgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -86,83 +102,33 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="6"/>
-      </left>
-      <right style="thin">
-        <color theme="6"/>
-      </right>
-      <top style="thin">
-        <color theme="6"/>
-      </top>
-      <bottom style="medium">
-        <color theme="6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -309,6 +275,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -343,6 +310,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -377,20 +345,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -512,7 +476,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -527,12 +530,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
@@ -565,298 +568,298 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>SUSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>SUTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>SUCAT</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>SUDOSE</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>SUDOSTXT</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>SUDOSU</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>SUDOSFRQ</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>SUSTDTC</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>SUENDTC</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>SUSTTPT</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>SUSTRTPT</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>SUENTPT</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>SUENRTPT</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Reported Name of Substance</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Category for Substance Use</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Substance Use Consumption</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Substance Use Consumption Text</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Consumption Units</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Use Frequency Per Interval</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Start Date/Time of Substance Use</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>End Date/Time of Substance Use</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Start Reference Time Point</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>Start Relative to Reference Time Point</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>End Reference Time Point</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>End Relative to Reference Time Point</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="P4" s="4" t="n">
+      <c r="H4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="P4" s="5" t="n">
         <v>50</v>
       </c>
     </row>
@@ -888,7 +891,7 @@
       <c r="G5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="6" t="n"/>
+      <c r="H5" s="6" t="str"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>PACK</t>
@@ -899,16 +902,20 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="M5" s="10" t="n">
-        <v>38718</v>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>2006-01-01</t>
+        </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>BEFORE</t>
         </is>
       </c>
-      <c r="O5" s="10" t="n">
-        <v>38718</v>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>2006-01-01</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -941,7 +948,7 @@
           <t>CAFFEINE</t>
         </is>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="10" t="n">
         <v>3</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -954,13 +961,13 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="K6" s="17" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>2006-01-
 01</t>
         </is>
       </c>
-      <c r="L6" s="17" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>2006-01-
 01</t>
@@ -1007,13 +1014,13 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="K7" s="17" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>2006-01-
 01</t>
         </is>
       </c>
-      <c r="L7" s="17" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>2006-01-
 01</t>
@@ -1035,12 +1042,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Filename</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
@@ -1141,39 +1148,145 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Error group</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Error level</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Row num</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Error value</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CMDOSTXT</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CMDOSTXT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ex.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>EXDOSTXT</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SUDOSTXT</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1191,244 +1304,244 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>AGSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>AGTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>AGPRESP</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>AGOCCUR</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>AGDOSE</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>AGDOSTXT</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>AGDOSU</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>AGROUTE</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>VISIT</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>AGENDTC</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Reported Agent Name</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>AG Pre-Specified</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>AG Occurrence</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Dose per Administration</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Dose Description</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Dose Units</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Route of Administration</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>Visit Name</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>End Date/Time of Agent</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
+      <c r="A4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
         <v>50</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1679,208 +1792,208 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>CMSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>CMTRT</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>CMDOSE</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>CMDOSTXT</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>CMDOSU</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>CMDOSFRQ</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>CMSTDTC</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>CMENDTC</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Reported Name of Drug, Med, or Therapy</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Dose per Administration</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Dose Description</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Dose Units</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Dosing Frequency per Interval</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Start Date/Time of Medication</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>End Date/Time of Medication</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="G4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1911,7 +2024,7 @@
       <c r="F5" t="n">
         <v>100</v>
       </c>
-      <c r="G5" s="6" t="n"/>
+      <c r="G5" s="6" t="str"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>mg</t>
@@ -1922,11 +2035,15 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="J5" s="7" t="n">
-        <v>37987</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>37989</v>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-01</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-03</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1953,7 +2070,7 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="10" t="n">
         <v>100</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -1966,11 +2083,15 @@
           <t>BID</t>
         </is>
       </c>
-      <c r="J6" s="7" t="n">
-        <v>37993</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>37993</v>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-07</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-07</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -2000,7 +2121,7 @@
       <c r="F7" t="n">
         <v>100</v>
       </c>
-      <c r="G7" s="6" t="n"/>
+      <c r="G7" s="6" t="str"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>mg</t>
@@ -2011,11 +2132,15 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="J7" s="9" t="n">
-        <v>37995</v>
-      </c>
-      <c r="K7" s="9" t="n">
-        <v>37995</v>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-09</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-09</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2042,7 +2167,7 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
@@ -2057,11 +2182,15 @@
           <t>PRN</t>
         </is>
       </c>
-      <c r="J8" s="7" t="n">
-        <v>37987</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>37995</v>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-01</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-09</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2106,11 +2235,15 @@
           <t>PRN</t>
         </is>
       </c>
-      <c r="J9" s="7" t="n">
-        <v>37987</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>37995</v>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-01</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-09</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2152,25 +2285,29 @@
           <t>BID</t>
         </is>
       </c>
-      <c r="J10" s="7" t="n">
-        <v>37987</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>37995</v>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-01</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-09</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="J11" s="10" t="n"/>
-      <c r="K11" s="10" t="n"/>
+      <c r="J11" s="6" t="str"/>
+      <c r="K11" s="6" t="str"/>
     </row>
     <row r="12"/>
     <row r="13">
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
+      <c r="I13" s="6" t="str"/>
+      <c r="J13" s="6" t="str"/>
     </row>
     <row r="14">
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
+      <c r="J14" s="6" t="str"/>
+      <c r="K14" s="6" t="str"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2183,378 +2320,530 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>STUDYID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>DOMAIN</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>ECSEQ</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>ECLNKID</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>ECTRT</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>ECREASOC</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>ECDOSE</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>ECDOSTXT</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>ECDOSU</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>ECDOSFRM</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>ECSTDTC</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>ECENDTC</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>ECSTDY</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>ECENDY</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="n"/>
-      <c r="B2" s="12" t="n"/>
-      <c r="C2" s="12" t="n"/>
-      <c r="D2" s="12" t="n"/>
-      <c r="E2" s="12" t="n"/>
-      <c r="F2" s="12" t="n"/>
-      <c r="G2" s="12" t="n"/>
-      <c r="H2" s="12" t="n"/>
-      <c r="I2" s="12" t="n"/>
-      <c r="J2" s="12" t="n"/>
-      <c r="K2" s="12" t="n"/>
-      <c r="L2" s="12" t="n"/>
-      <c r="M2" s="12" t="n"/>
-      <c r="N2" s="12" t="n"/>
-      <c r="O2" s="12" t="n"/>
-      <c r="P2" s="12" t="n"/>
-      <c r="Q2" s="12" t="n"/>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Study Identifier</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Domain Abbreviation</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Unique Subject Identifier</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Sequence Number</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Link ID</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Name of Treatment</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Pre-Specified</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Occurrence</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Reason for Occur Value</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Dose</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>Dose Description</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>Dose Units</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>Dose Form</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t>Start Date/Time of Treatment</t>
+        </is>
+      </c>
+      <c r="O2" s="8" t="inlineStr">
+        <is>
+          <t>End Date/Time of Treatment</t>
+        </is>
+      </c>
+      <c r="P2" s="8" t="inlineStr">
+        <is>
+          <t>Study Day of Start of Treatment</t>
+        </is>
+      </c>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>Study Day of End of Treatment</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n"/>
-      <c r="B3" s="12" t="n"/>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="n"/>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="n"/>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="n"/>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-      <c r="P3" s="12" t="n"/>
-      <c r="Q3" s="12" t="n"/>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>STUDYID</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>DOMAIN</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>USUBJID</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>ECSEQ</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>ECLNKID</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>ECTRT</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>ECPRESP</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>ECOCCUR</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>ECREASOC</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSE</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSTXT</t>
-        </is>
-      </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSU</t>
-        </is>
-      </c>
-      <c r="M4" s="13" t="inlineStr">
-        <is>
-          <t>ECDOSFRM</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>ECSTDTC</t>
-        </is>
-      </c>
-      <c r="O4" s="13" t="inlineStr">
-        <is>
-          <t>ECENDTC</t>
-        </is>
-      </c>
-      <c r="P4" s="13" t="inlineStr">
-        <is>
-          <t>ECSTDY</t>
-        </is>
-      </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>ECENDY</t>
-        </is>
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="P4" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="8" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Study Identifier</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Domain Abbreviation</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Unique Subject Identifier</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Sequence Number</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>Link ID</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>Name of Treatment</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>Pre-Specified</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>Occurrence</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>Reason for Occur Value</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="inlineStr">
-        <is>
-          <t>Dose</t>
-        </is>
-      </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>Dose Description</t>
-        </is>
-      </c>
-      <c r="L5" s="14" t="inlineStr">
-        <is>
-          <t>Dose Units</t>
-        </is>
-      </c>
-      <c r="M5" s="14" t="inlineStr">
-        <is>
-          <t>Dose Form</t>
-        </is>
-      </c>
-      <c r="N5" s="14" t="inlineStr">
-        <is>
-          <t>Start Date/Time of Treatment</t>
-        </is>
-      </c>
-      <c r="O5" s="14" t="inlineStr">
-        <is>
-          <t>End Date/Time of Treatment</t>
-        </is>
-      </c>
-      <c r="P5" s="14" t="inlineStr">
-        <is>
-          <t>Study Day of Start of Treatment</t>
-        </is>
-      </c>
-      <c r="Q5" s="14" t="inlineStr">
-        <is>
-          <t>Study Day of End of Treatment</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ABC1001</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A2-20110114</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>TABLET</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-14</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-28</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="O6" s="14" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="P6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="Q6" s="14" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ABC2001</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A2-20110114</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>TABLET</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-14</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-23</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="H7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="I7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="J7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="L7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="M7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="N7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="O7" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="P7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q7" s="14" t="n">
-        <v>8</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ABC2001</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A0-20110124</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>PATIENT MISTAKE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>TABLET</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-24</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-24</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -2570,15 +2859,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ABC1001</t>
+          <t>ABC2001</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A2-20110114</t>
+          <t>A2-20110125</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2609,213 +2898,20 @@
           <t>QD</t>
         </is>
       </c>
-      <c r="N8" s="10" t="n">
-        <v>40557</v>
-      </c>
-      <c r="O8" s="10" t="n">
-        <v>40571</v>
+      <c r="N8" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-25</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-28</t>
+        </is>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="Q8" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ABC2001</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>A2-20110114</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>BOTTLE A</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>QD</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="n">
-        <v>40557</v>
-      </c>
-      <c r="O9" s="10" t="n">
-        <v>40566</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>ABC2001</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>A0-20110124</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>BOTTLE A</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>PATIENT MISTAKE</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>QD</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="n">
-        <v>40567</v>
-      </c>
-      <c r="O10" s="10" t="n">
-        <v>40567</v>
-      </c>
-      <c r="P10" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>EC</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>ABC2001</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>A2-20110125</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>BOTTLE A</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>QD</t>
-        </is>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>40568</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>40571</v>
-      </c>
-      <c r="P11" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q11" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2834,298 +2930,298 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>EXSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>EXLNKID</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>EXTRT</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>EXDOSE</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>EXDOSTXT</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>EXDOSU</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>EXDOSFRM</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>EXDOSFRQ</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>EXROUTE</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>EXSTDTC</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>EXENDTC</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>EXSTDY</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>EXENDY</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Link ID</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Name of Treatment</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Dose</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Dose Description</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Dose Units</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Dose Form</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Dosing Frequency per Interval</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>Route of Administration</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Start Date/Time of Treatment</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>End Date/Time of Treatment</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Study Day of Start of Treatment</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>Study Day of End of Treatment</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" s="4" t="n">
+      <c r="H4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="5" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3181,11 +3277,15 @@
           <t>ORAL</t>
         </is>
       </c>
-      <c r="M5" s="10" t="n">
-        <v>40557</v>
-      </c>
-      <c r="N5" s="10" t="n">
-        <v>40571</v>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-14</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-28</t>
+        </is>
       </c>
       <c r="O5" t="n">
         <v>1</v>
@@ -3223,7 +3323,7 @@
           <t>DRUG Z</t>
         </is>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="10" t="n">
         <v>500</v>
       </c>
       <c r="I6" t="inlineStr">
@@ -3246,11 +3346,15 @@
           <t>ORAL</t>
         </is>
       </c>
-      <c r="M6" s="10" t="n">
-        <v>40557</v>
-      </c>
-      <c r="N6" s="10" t="n">
-        <v>40566</v>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-14</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-23</t>
+        </is>
       </c>
       <c r="O6" t="n">
         <v>1</v>
@@ -3311,11 +3415,15 @@
           <t>ORAL</t>
         </is>
       </c>
-      <c r="M7" s="10" t="n">
-        <v>40568</v>
-      </c>
-      <c r="N7" s="10" t="n">
-        <v>40571</v>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-25</t>
+        </is>
+      </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>2011-01-28</t>
+        </is>
       </c>
       <c r="O7" t="n">
         <v>12</v>
@@ -3339,316 +3447,316 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>MLSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>MLTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>MLCAT</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>MLPRESP</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>MLOCCUR</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>MLDOSE</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>MLDOSTXT</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>MLDOSU</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>MLDTC</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>MLSTDTC</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>MLENDTC</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>RELMIDS</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>MIDS</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>MIDSDTC</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Name of Meal</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Category for Meal</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>ML Pre-specified</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>ML Occurrence</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Dose</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Dose Description</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Dose Units</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>Date/Time of Collection</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Start Date/Time of Meal</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>End Date/Time of Meal</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Temporal Relation to Milestone Instance</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>Disease Milestone Instance Name</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>Disease Milestone Instance Date/Time</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="4" t="n">
+      <c r="J4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="5" t="n">
         <v>50</v>
       </c>
     </row>
@@ -3696,7 +3804,7 @@
           <t>2015-06-03T14:15</t>
         </is>
       </c>
-      <c r="O5" s="16" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>LAST
 MEAL
@@ -3734,7 +3842,7 @@
       <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>NUTRITIONAL
 DRINK</t>
@@ -3765,13 +3873,13 @@
           <t>oz</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>2015-09-
 03T08:30</t>
         </is>
       </c>
-      <c r="O6" s="16" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>LAST
 MEAL
@@ -3784,7 +3892,7 @@
           <t>HYPO2</t>
         </is>
       </c>
-      <c r="Q6" s="16" t="inlineStr">
+      <c r="Q6" s="6" t="inlineStr">
         <is>
           <t>2015-09-
 03T17:00</t>
@@ -3806,226 +3914,226 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>PRSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>PRTRT</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>PRDOSE</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>PRDOSTXT</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>PRDOSU</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>PRLOC</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>PRLAT</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>PRSTDTC</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>PRENDTC</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Reported Name of Procedure</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Dose</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Dose Description</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Dose Units</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>Location of Procedure</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Laterality</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Start Date/Time of Procedure</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>End Date/Time of Procedure</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
+      <c r="E4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="G4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="n">
         <v>50</v>
       </c>
     </row>
@@ -4071,11 +4179,15 @@
           <t>RIGHT</t>
         </is>
       </c>
-      <c r="K5" s="10" t="n">
-        <v>40695</v>
-      </c>
-      <c r="L5" s="10" t="n">
-        <v>40719</v>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>2011-06-01</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>2011-06-25</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -4117,11 +4229,15 @@
           <t>PROSTATE</t>
         </is>
       </c>
-      <c r="K6" s="10" t="n">
-        <v>40739</v>
-      </c>
-      <c r="L6" s="10" t="n">
-        <v>40739</v>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>2011-07-15</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>2011-07-15</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -4161,11 +4277,15 @@
           <t>BONE</t>
         </is>
       </c>
-      <c r="K7" s="10" t="n">
-        <v>40774</v>
-      </c>
-      <c r="L7" s="10" t="n">
-        <v>40777</v>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>2011-08-19</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>2011-08-22</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added --TRT and --DOSTXT output variables, update test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000094/negative/01/data/unit-test-coreid-CG0112-negative.xlsx
+++ b/rules/CORE-000094/negative/01/data/unit-test-coreid-CG0112-negative.xlsx
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -124,6 +124,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -938,7 +939,7 @@
       <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>COFFEE</t>
         </is>
@@ -1148,7 +1149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1202,16 +1203,18 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CMDOSTXT</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>100</v>
+          <t>CMTRT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ASPIRIN</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1224,26 +1227,24 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>CMDOSTXT</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
+      <c r="F3" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ex.xpt</t>
+          <t>cm.xpt</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1252,40 +1253,152 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>EXDOSTXT</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>500</v>
+          <t>CMTRT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ASPIRIN</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CMDOSTXT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ex.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>EXTRT</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>DRUG Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ex.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>EXDOSTXT</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>su.xpt</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Record</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D8" t="n">
         <v>6</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SUTRT</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>COFFEE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>SUDOSTXT</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F9" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2065,7 +2178,7 @@
       <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>ASPIRIN</t>
         </is>
@@ -2162,7 +2275,7 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>ASPIRIN</t>
         </is>
@@ -2300,7 +2413,6 @@
       <c r="J11" s="6" t="str"/>
       <c r="K11" s="6" t="str"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="I13" s="6" t="str"/>
       <c r="J13" s="6" t="str"/>
@@ -3318,7 +3430,7 @@
           <t>A2-20110114</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>DRUG Z</t>
         </is>

</xml_diff>

<commit_message>
CORE-000094: allow optional leading minus in --DOSTXT numeric regex
Per review comment, the matches_regex pattern now also flags negative
numbers (e.g. "-5") as numeric --DOSTXT values, guarding against
mistaken entries even though doses can't logically be negative. Added
a negative test case in cm.xpt to cover it.
</commit_message>
<xml_diff>
--- a/rules/CORE-000094/negative/01/data/unit-test-coreid-CG0112-negative.xlsx
+++ b/rules/CORE-000094/negative/01/data/unit-test-coreid-CG0112-negative.xlsx
@@ -1149,7 +1149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1400,6 +1400,62 @@
       </c>
       <c r="F9" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CMTRT</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ASPIRIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>11</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CMDOSTXT</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2410,8 +2466,54 @@
       </c>
     </row>
     <row r="11">
-      <c r="J11" s="6" t="str"/>
-      <c r="K11" s="6" t="str"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ABC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ABC-0005</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>ASPIRIN</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>QD</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-01</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>2004-01-09</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="I13" s="6" t="str"/>

</xml_diff>